<commit_message>
Add DP validation to bulk import; update fixture dp_shares to -15000
- bulk_create_grants now validates each grant's dp_shares against
  existing DB grants + other grants in the batch
- fixture: 2024 Purchase dp_shares -2000 → -15000 (~10% of grant,
  more realistic than 1.3%)
- Known-good values updated: cum_shares 571500→558500,
  cum_cap_gains 1243695→1224195 (13k fewer shares × subsequent
  price increases of $0.65 + $0.85)

https://claude.ai/code/session_01WBWRojrJEDx97JdfuAYKzt
</commit_message>
<xml_diff>
--- a/test_data/fixture.xlsx
+++ b/test_data/fixture.xlsx
@@ -18,12 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -451,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="5" max="5"/>
@@ -1052,7 +1051,7 @@
         <v>45657</v>
       </c>
       <c r="H12" t="n">
-        <v>-2000</v>
+        <v>-15000</v>
       </c>
       <c r="I12">
         <f>C12-H12</f>
@@ -1127,7 +1126,6 @@
       <c r="N13" s="12" t="n"/>
       <c r="O13" s="2" t="n"/>
     </row>
-    <row r="14"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>